<commit_message>
Committing one missing file from variant update
</commit_message>
<xml_diff>
--- a/src_files/data_files/Finland_dheat_and_industry.xlsx
+++ b/src_files/data_files/Finland_dheat_and_industry.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BB\bb-dev\north_european_model\src_files\data_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29F0085C-5ECF-4632-AA00-904CB7428DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA837C2F-6AF6-40FC-8224-3C6BA4409693}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="889" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5159,9 +5159,6 @@
     <t>cities</t>
   </si>
   <si>
-    <t>every city its own node</t>
-  </si>
-  <si>
     <t>capitals</t>
   </si>
   <si>
@@ -5202,6 +5199,9 @@
   </si>
   <si>
     <t>capital region, rest of the country</t>
+  </si>
+  <si>
+    <t>major cities separately</t>
   </si>
 </sst>
 </file>
@@ -58597,7 +58597,7 @@
         <v>2</v>
       </c>
       <c r="H1" s="92" t="s">
-        <v>1681</v>
+        <v>1680</v>
       </c>
       <c r="I1" s="92" t="s">
         <v>1609</v>
@@ -59630,7 +59630,7 @@
         <v>1606</v>
       </c>
       <c r="V1" t="s">
-        <v>1682</v>
+        <v>1681</v>
       </c>
       <c r="W1" t="s">
         <v>1619</v>
@@ -59692,7 +59692,7 @@
     </row>
     <row r="2" spans="1:41">
       <c r="A2" s="106" t="s">
-        <v>1686</v>
+        <v>1685</v>
       </c>
       <c r="B2" s="106"/>
       <c r="C2" s="106"/>
@@ -59923,7 +59923,7 @@
         <v>1678</v>
       </c>
       <c r="X5" s="104" t="s">
-        <v>1680</v>
+        <v>1679</v>
       </c>
       <c r="AA5" t="s">
         <v>1620</v>
@@ -65821,7 +65821,7 @@
     </row>
     <row r="80" spans="1:22">
       <c r="A80" s="106" t="s">
-        <v>1692</v>
+        <v>1691</v>
       </c>
       <c r="B80" s="106"/>
       <c r="C80" s="106"/>
@@ -66027,7 +66027,7 @@
     </row>
     <row r="84" spans="1:19">
       <c r="A84" s="106" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="B84" s="106"/>
       <c r="C84" s="106"/>
@@ -66194,7 +66194,7 @@
     </row>
     <row r="93" spans="1:19">
       <c r="A93" s="106" t="s">
-        <v>1684</v>
+        <v>1683</v>
       </c>
       <c r="B93" s="106"/>
       <c r="C93" s="106"/>
@@ -68015,7 +68015,7 @@
     </row>
     <row r="123" spans="1:19">
       <c r="A123" s="106" t="s">
-        <v>1685</v>
+        <v>1684</v>
       </c>
       <c r="B123" s="106"/>
       <c r="C123" s="106"/>
@@ -68050,7 +68050,7 @@
         <v>1</v>
       </c>
       <c r="F124" s="53" t="s">
-        <v>1687</v>
+        <v>1686</v>
       </c>
       <c r="G124" s="108">
         <f ca="1">SUMIFS(G$94:G$122,$B$94:$B$122,$B124)</f>
@@ -68079,7 +68079,7 @@
         <v>1</v>
       </c>
       <c r="F125" s="53" t="s">
-        <v>1687</v>
+        <v>1686</v>
       </c>
       <c r="G125" s="108">
         <f t="shared" ref="G125:K139" ca="1" si="27">SUMIFS(G$94:G$122,$B$94:$B$122,$B125)</f>
@@ -68108,7 +68108,7 @@
         <v>1</v>
       </c>
       <c r="F126" s="53" t="s">
-        <v>1687</v>
+        <v>1686</v>
       </c>
       <c r="G126" s="108">
         <f t="shared" ca="1" si="27"/>
@@ -68137,7 +68137,7 @@
         <v>1</v>
       </c>
       <c r="F127" s="53" t="s">
-        <v>1687</v>
+        <v>1686</v>
       </c>
       <c r="G127" s="108">
         <f t="shared" ca="1" si="27"/>
@@ -68166,7 +68166,7 @@
         <v>1</v>
       </c>
       <c r="F128" s="53" t="s">
-        <v>1687</v>
+        <v>1686</v>
       </c>
       <c r="G128" s="108">
         <f t="shared" ca="1" si="27"/>
@@ -68195,7 +68195,7 @@
         <v>1</v>
       </c>
       <c r="F129" s="53" t="s">
-        <v>1687</v>
+        <v>1686</v>
       </c>
       <c r="G129" s="108">
         <f t="shared" ca="1" si="27"/>
@@ -68224,7 +68224,7 @@
         <v>1</v>
       </c>
       <c r="F130" s="53" t="s">
-        <v>1687</v>
+        <v>1686</v>
       </c>
       <c r="G130" s="108">
         <f t="shared" ca="1" si="27"/>
@@ -68253,7 +68253,7 @@
         <v>1</v>
       </c>
       <c r="F131" s="53" t="s">
-        <v>1687</v>
+        <v>1686</v>
       </c>
       <c r="G131" s="108">
         <f t="shared" ca="1" si="27"/>
@@ -68282,7 +68282,7 @@
         <v>1</v>
       </c>
       <c r="F132" s="53" t="s">
-        <v>1687</v>
+        <v>1686</v>
       </c>
       <c r="G132" s="108">
         <f t="shared" ca="1" si="27"/>
@@ -68311,7 +68311,7 @@
         <v>1</v>
       </c>
       <c r="F133" s="53" t="s">
-        <v>1687</v>
+        <v>1686</v>
       </c>
       <c r="G133" s="108">
         <f t="shared" ca="1" si="27"/>
@@ -68340,7 +68340,7 @@
         <v>1</v>
       </c>
       <c r="F134" s="53" t="s">
-        <v>1687</v>
+        <v>1686</v>
       </c>
       <c r="G134" s="108">
         <f t="shared" ca="1" si="27"/>
@@ -68369,7 +68369,7 @@
         <v>1</v>
       </c>
       <c r="F135" s="53" t="s">
-        <v>1687</v>
+        <v>1686</v>
       </c>
       <c r="G135" s="108">
         <f t="shared" ca="1" si="27"/>
@@ -68398,7 +68398,7 @@
         <v>1</v>
       </c>
       <c r="F136" s="53" t="s">
-        <v>1687</v>
+        <v>1686</v>
       </c>
       <c r="G136" s="108">
         <f t="shared" ca="1" si="27"/>
@@ -68427,7 +68427,7 @@
         <v>1</v>
       </c>
       <c r="F137" s="53" t="s">
-        <v>1687</v>
+        <v>1686</v>
       </c>
       <c r="G137" s="108">
         <f t="shared" ca="1" si="27"/>
@@ -68456,7 +68456,7 @@
         <v>1</v>
       </c>
       <c r="F138" s="53" t="s">
-        <v>1687</v>
+        <v>1686</v>
       </c>
       <c r="G138" s="108">
         <f t="shared" ca="1" si="27"/>
@@ -68485,7 +68485,7 @@
         <v>1</v>
       </c>
       <c r="F139" s="53" t="s">
-        <v>1687</v>
+        <v>1686</v>
       </c>
       <c r="G139" s="108">
         <f t="shared" ca="1" si="27"/>
@@ -68502,7 +68502,7 @@
     </row>
     <row r="143" spans="1:11">
       <c r="A143" t="s">
-        <v>1688</v>
+        <v>1687</v>
       </c>
       <c r="B143" t="s">
         <v>4</v>
@@ -68516,7 +68516,7 @@
     </row>
     <row r="144" spans="1:11">
       <c r="A144" t="s">
-        <v>1689</v>
+        <v>1688</v>
       </c>
       <c r="B144">
         <f ca="1">SUM(G3:G79)</f>
@@ -68533,7 +68533,7 @@
     </row>
     <row r="145" spans="1:4">
       <c r="A145" t="s">
-        <v>1690</v>
+        <v>1689</v>
       </c>
       <c r="B145">
         <f ca="1">SUM(G94:G122)</f>
@@ -68550,7 +68550,7 @@
     </row>
     <row r="146" spans="1:4">
       <c r="A146" t="s">
-        <v>1691</v>
+        <v>1690</v>
       </c>
       <c r="B146">
         <f ca="1">SUM(G124:G139)</f>
@@ -68621,7 +68621,7 @@
         <v>1673</v>
       </c>
       <c r="B3" t="s">
-        <v>1680</v>
+        <v>1679</v>
       </c>
       <c r="C3" t="s">
         <v>1675</v>
@@ -68630,7 +68630,7 @@
         <v>1676</v>
       </c>
       <c r="E3" t="s">
-        <v>1693</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -68644,7 +68644,7 @@
         <v>1676</v>
       </c>
       <c r="E4" t="s">
-        <v>1679</v>
+        <v>1693</v>
       </c>
     </row>
   </sheetData>

</xml_diff>